<commit_message>
data(galactic-baseballer): G16-P4-B2 audit reference boundaries
</commit_message>
<xml_diff>
--- a/config/galactic-baseballer-generated/templates/GalacticBaseballerProfiles.xlsx
+++ b/config/galactic-baseballer-generated/templates/GalacticBaseballerProfiles.xlsx
@@ -57,7 +57,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>863e22a454bacb9d</t>
+    <t>4455928244bfecda</t>
   </si>
   <si>
     <t>#name</t>
@@ -1431,7 +1431,7 @@
         <v>41</v>
       </c>
       <c r="AA4" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AB4" s="5" t="s">
         <v>41</v>

</xml_diff>